<commit_message>
EPBDS-16811 Fix SmartRules and SimpleRules turning an integer column into ranges when a numeric cell is beyond the int range
</commit_message>
<xml_diff>
--- a/DEV/org.openl.rules/test/rules/dt/BigIntegerConditions.xlsx
+++ b/DEV/org.openl.rules/test/rules/dt/BigIntegerConditions.xlsx
@@ -7,12 +7,13 @@
   </bookViews>
   <sheets>
     <sheet name="Ranges" r:id="rId3" sheetId="1"/>
+    <sheet name="Numbers" r:id="rId4" sheetId="2"/>
   </sheets>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="10">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="17">
   <si>
     <t>SmartRules String bigIntegerInRanges(BigInteger value)</t>
   </si>
@@ -42,6 +43,27 @@
   </si>
   <si>
     <t>SimpleRules String longInRangesSimple(Long value)</t>
+  </si>
+  <si>
+    <t>SmartRules String bigIntegerNumbers(BigInteger value)</t>
+  </si>
+  <si>
+    <t>int max</t>
+  </si>
+  <si>
+    <t>beyond int</t>
+  </si>
+  <si>
+    <t>beyond long</t>
+  </si>
+  <si>
+    <t>SimpleRules String bigIntegerNumbersSimple(BigInteger value)</t>
+  </si>
+  <si>
+    <t>SmartRules String longNumbers(Long value)</t>
+  </si>
+  <si>
+    <t>SimpleRules String longNumbersSimple(Long value)</t>
   </si>
 </sst>
 </file>
@@ -208,4 +230,146 @@
   </sheetData>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1:B21"/>
+  <sheetFormatPr defaultRowHeight="15.0"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="s" s="0">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="s" s="0">
+        <v>1</v>
+      </c>
+      <c r="B2" t="s" s="0">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n" s="0">
+        <v>2.147483647E9</v>
+      </c>
+      <c r="B3" t="s" s="0">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n" s="0">
+        <v>2.147483648E9</v>
+      </c>
+      <c r="B4" t="s" s="0">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n" s="0">
+        <v>1.0E20</v>
+      </c>
+      <c r="B5" t="s" s="0">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="s" s="0">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="s" s="0">
+        <v>1</v>
+      </c>
+      <c r="B8" t="s" s="0">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n" s="0">
+        <v>2.147483647E9</v>
+      </c>
+      <c r="B9" t="s" s="0">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n" s="0">
+        <v>2.147483648E9</v>
+      </c>
+      <c r="B10" t="s" s="0">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n" s="0">
+        <v>1.0E20</v>
+      </c>
+      <c r="B11" t="s" s="0">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="s" s="0">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="s" s="0">
+        <v>1</v>
+      </c>
+      <c r="B14" t="s" s="0">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n" s="0">
+        <v>2.147483647E9</v>
+      </c>
+      <c r="B15" t="s" s="0">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n" s="0">
+        <v>2.147483648E9</v>
+      </c>
+      <c r="B16" t="s" s="0">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="s" s="0">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="s" s="0">
+        <v>1</v>
+      </c>
+      <c r="B19" t="s" s="0">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="n" s="0">
+        <v>2.147483647E9</v>
+      </c>
+      <c r="B20" t="s" s="0">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="n" s="0">
+        <v>2.147483648E9</v>
+      </c>
+      <c r="B21" t="s" s="0">
+        <v>12</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
+</worksheet>
 </file>
</xml_diff>